<commit_message>
Add scouting shortlist by archetype, capped at 10 per group
New Shortlist sheet in the workbook: top 10 players per Primary
Archetype ranked by Scouting Score, with Uncertainty Score and
Confidence alongside each name. Also ships as a standalone visual
(Shortlist_ByArchetype.png) with a mini scouting-score bar and a
confidence-colored uncertainty dot per player.

Caught and fixed a real contrast bug while verifying in dark mode: the
Uncertainty numbers were rendering in near-black text on the dark
surface (invisible), while Scouting numbers were fine, because the
uncertainty cell never got an explicit text color and something in
the inheritance chain broke for that element specifically. Added an
explicit color rule to fix it.
</commit_message>
<xml_diff>
--- a/reports/Japan_Strikers_Scouting.xlsx
+++ b/reports/Japan_Strikers_Scouting.xlsx
@@ -8,13 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Strikers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Uncertainty" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Archetype Z" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Methodology" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Shortlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Uncertainty" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Archetype Z" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Methodology" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Strikers'!$A$1:$O$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Uncertainty'!$A$1:$H$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shortlist'!$A$1:$J$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Uncertainty'!$A$1:$H$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,7 +38,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +48,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001D4ED8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,11 +68,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4742,6 +4750,1873 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Primary Archetype</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Minutes</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Scouting Score</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Uncertainty Score</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>R. Arita</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Kagoshima United</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F2" t="n">
+        <v>885</v>
+      </c>
+      <c r="G2" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Very Good Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>D. Furukawa</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Renofa Yamaguchi</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>26</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1177</v>
+      </c>
+      <c r="G3" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>T. Nakashima</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Thespa Gunma</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1001</v>
+      </c>
+      <c r="G4" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Patric</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Zweigen Kanazawa</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F5" t="n">
+        <v>733</v>
+      </c>
+      <c r="G5" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="H5" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Low confidence</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>K. Sagawa</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Blaublitz Akita</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1020</v>
+      </c>
+      <c r="G6" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Matheus Peixoto</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Júbilo Iwata</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1104</v>
+      </c>
+      <c r="G7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>K. Buwanika</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Zweigen Kanazawa</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>23</v>
+      </c>
+      <c r="F8" t="n">
+        <v>918</v>
+      </c>
+      <c r="G8" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>R. Ota</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ventforet Kofu</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" t="n">
+        <v>967</v>
+      </c>
+      <c r="G9" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>T. Kato</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Matsumoto Yamaga</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>26</v>
+      </c>
+      <c r="F10" t="n">
+        <v>952</v>
+      </c>
+      <c r="G10" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>26</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Solid Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Target Striker</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>K. Watanabe</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Shonan Bellmare</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>23</v>
+      </c>
+      <c r="F11" t="n">
+        <v>883</v>
+      </c>
+      <c r="G11" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="H11" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Fringe Target Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Lucas Barcelos</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Tokushima Vortis</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>1192</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>K. Tsuboi</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Kataller Toyama</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>766</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>H. Iwabuchi</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Vegalta Sendai</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>1068</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Y. Taguchi</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Ehime</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>954</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>69.09999999999999</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>S. Tamura</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Nara Club</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>1409</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Solid Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Y. Toshida</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Tegevajaro Miyazaki</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>1286</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Solid Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>A. Bakayoko</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Consadole Sapporo</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>722</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Solid Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>M. Shintani</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Kochi United</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>1225</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Solid Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>S. Omori</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Consadole Sapporo</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>735</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Solid Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Goalscoring Striker</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>H. Yamada</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Shonan Bellmare</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>1195</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Solid Goalscoring Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Thonny Anderson</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tokushima Vortis</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>28</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G22" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Very Good Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Edigar Junio</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Imabari</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>35</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1138</v>
+      </c>
+      <c r="G23" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Solid Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>K. Murakoshi</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Matsumoto Yamaga</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>24</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1564</v>
+      </c>
+      <c r="G24" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Solid Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Y. Nishimura</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Thespa Gunma</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>26</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1378</v>
+      </c>
+      <c r="G25" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>H. Asakawa</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Ryūkyū</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>31</v>
+      </c>
+      <c r="F26" t="n">
+        <v>892</v>
+      </c>
+      <c r="G26" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>T. Kitsui</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>33</v>
+      </c>
+      <c r="F27" t="n">
+        <v>996</v>
+      </c>
+      <c r="G27" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="H27" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>K. Kawamura</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Kagoshima United</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>26</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1348</v>
+      </c>
+      <c r="G28" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="H28" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>R. Watanabe</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Júbilo Iwata</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>29</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1054</v>
+      </c>
+      <c r="G29" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>9</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A. Inoue</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Matsumoto Yamaga</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>19</v>
+      </c>
+      <c r="F30" t="n">
+        <v>721</v>
+      </c>
+      <c r="G30" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Second Striker</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>K. Fujikawa</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Parceiro Nagano</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>27</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1208</v>
+      </c>
+      <c r="G31" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="H31" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Fringe Second Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Matheus Moraes</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Albirex Niigata</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>917</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>R. Kawamoto</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Gifu</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>1558</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>R. Shiohama</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Sagan Tosu</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Very Good Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Gustavo Silva</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Júbilo Iwata</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>1086</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Solid Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>K. Mori</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Imabari</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>916</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Solid Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Y. Wakatsuki</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Albirex Niigata</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>1096</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Solid Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>T. Kato</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Iwaki</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>941</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Fringe Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>K. Kasai</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Albirex Niigata</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>1123</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>High confidence</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Fringe Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>M. Handai</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Roasso Kumamoto</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>722</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Fringe Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Striker</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>K. Hoshi</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Gainare Tottori</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>945</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Fringe Dynamic Striker</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Complete Forward</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>T. Nishino</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Tochigi SC</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>23</v>
+      </c>
+      <c r="F42" t="n">
+        <v>800</v>
+      </c>
+      <c r="G42" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="H42" t="n">
+        <v>30</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Elite Complete Forward</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Complete Forward</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>K. Shimizu</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Fukushima United</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>24</v>
+      </c>
+      <c r="F43" t="n">
+        <v>852</v>
+      </c>
+      <c r="G43" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="H43" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Medium confidence</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Elite Complete Forward</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J43"/>
+  <conditionalFormatting sqref="G2:G43">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F87171"/>
+        <color rgb="00FEF08A"/>
+        <color rgb="004ADE80"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H43">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="004ADE80"/>
+        <color rgb="00FEF08A"/>
+        <color rgb="00F87171"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6975,7 +8850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13001,7 +14876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Split scouting shortlist into 4 per-archetype images, drop Complete Forward
Replaces the single combined shortlist grid with one standalone image
per archetype (Target, Goalscoring, Second, Dynamic Striker), each
carrying its own title and footnote. Complete Forward is excluded from
the shortlist entirely (both the visuals and the workbook's Shortlist
sheet) since it's a 2-player edge case, not a real target pool.
</commit_message>
<xml_diff>
--- a/reports/Japan_Strikers_Scouting.xlsx
+++ b/reports/Japan_Strikers_Scouting.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Strikers'!$A$1:$O$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shortlist'!$A$1:$J$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shortlist'!$A$1:$J$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Uncertainty'!$A$1:$H$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4750,7 +4750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6497,93 +6497,9 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Complete Forward</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>T. Nishino</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Tochigi SC</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>23</v>
-      </c>
-      <c r="F42" t="n">
-        <v>800</v>
-      </c>
-      <c r="G42" t="n">
-        <v>89.8</v>
-      </c>
-      <c r="H42" t="n">
-        <v>30</v>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Medium confidence</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Elite Complete Forward</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Complete Forward</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>K. Shimizu</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Fukushima United</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>24</v>
-      </c>
-      <c r="F43" t="n">
-        <v>852</v>
-      </c>
-      <c r="G43" t="n">
-        <v>80.40000000000001</v>
-      </c>
-      <c r="H43" t="n">
-        <v>39.8</v>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Medium confidence</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Elite Complete Forward</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J43"/>
-  <conditionalFormatting sqref="G2:G43">
+  <autoFilter ref="A1:J41"/>
+  <conditionalFormatting sqref="G2:G41">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -6595,7 +6511,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H43">
+  <conditionalFormatting sqref="H2:H41">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>